<commit_message>
added rest assure framework changes
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rkuma\SeleniumGitWFProject\LatestProject\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{962458E9-337D-4F7A-80D8-C2D0785BA907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A0BC017-4ED9-44BE-A9A2-9241FBC23BF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="RestAssured" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="10">
   <si>
     <t>ScenarioName</t>
   </si>
@@ -37,19 +38,43 @@
   </si>
   <si>
     <t>Mobiles</t>
+  </si>
+  <si>
+    <t>Scenario_AddBook</t>
+  </si>
+  <si>
+    <t>Step01</t>
+  </si>
+  <si>
+    <t>StepNo</t>
+  </si>
+  <si>
+    <t>Step02</t>
+  </si>
+  <si>
+    <t>Step03</t>
+  </si>
+  <si>
+    <t>Scenario</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -72,8 +97,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -376,4 +403,60 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{248F7C75-4CE4-4C7B-B864-106247C59D8E}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18.5546875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="20.109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="41.88671875" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.88671875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>